<commit_message>
Restrict each bucket to the cost types the Standard describes for it; add the cost-type by bucket matrix to the month report
Dentist pay no longer enters the Laboratory or Prosthesis buckets; nurses may
sit in Dental, Imaging and Anaesthesia; overheads only in Dental. The engine
writes the fitted bucket x cost-type matrix and the report shows it in AED.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/output/January_Model_Report.xlsx
+++ b/output/January_Model_Report.xlsx
@@ -10,10 +10,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost types" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buckets" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bucket profiles" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implant claims" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim examples" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Type x Bucket" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bucket profiles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implant claims" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim examples" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -63,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -71,6 +72,8 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1191,6 +1194,531 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Cost type (WHAT)</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Anaesthesia</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Dental</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Imaging</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Prosthesis</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Ledger</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Share in Dental</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SWNurs</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>1545.928</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>14629.143</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>8924.929</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>25100</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>25100</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0.5828343824701195</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SWDoc</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>20053.877</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>151816.123</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>171870</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>171870</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0.8833195031128178</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SWAllied</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>1318.135</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>1608.333</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>11223.532</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>14150</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>14150</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0.09315441696113075</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>47.998</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>13622.816</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>3608.126</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>17278.94</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>17278.94</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0.002777832436480478</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>1143.765</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>108.235</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>1252</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>1252</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>0.08644968051118211</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Prostheses</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>52796</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>52796</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>52796</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>626.178</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>3950.357</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>964.0119999999999</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>11212.039</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>62.112</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>14848.052</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>31662.75</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>31662.75</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0.1247635470702955</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>888.27</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>111.73</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0.88827</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Depreciation</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>2086.95</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>2546.407</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>5923.253</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>10556.61</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>10556.61</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0.1976913043107588</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>174794.2</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>174794.2</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>174794.2</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OHDepreciation</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OHC</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>8317</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>8317</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>8317</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL (WHERE)</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>23369.748</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>360481.211</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>14043.681</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>41981.64</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>173.842</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>71252.178</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>511302.3</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>511302.3</v>
+      </c>
+      <c r="J14" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Read across a row: where that cost type sits (buckets). Read down a column: what that bucket is made of (cost types). Both add to the month ledger.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1218,7 +1746,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SWDoc 81.3%, Pharmacy 5.0%, MS 13.8%</t>
+          <t>SWNurs 6.6%, SWDoc 85.8%, Pharmacy 4.9%, MS 2.7%</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1758,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SWNurs 6.1%, SWDoc 33.8%, SWAllied 1.7%, Laboratory 0.1%, Pharmacy 0.0%, MS 4.8%, GS 0.3%, Depreciation 1.7%, OHF 48.5%, OHDepreciation 0.7%, OHC 2.3%</t>
+          <t>SWNurs 4.1%, SWDoc 42.1%, SWAllied 0.4%, Laboratory 0.0%, Pharmacy 0.0%, MS 1.1%, GS 0.2%, Depreciation 0.6%, OHF 48.5%, OHDepreciation 0.7%, OHC 2.3%</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1770,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SWNurs 21.7%, SWAllied 30.6%, MS 16.9%, Depreciation 30.7%</t>
+          <t>SWNurs 63.6%, SWAllied 11.5%, MS 6.9%, Depreciation 18.1%</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1782,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SWDoc 42.7%, SWAllied 8.7%, Laboratory 36.5%, MS 12.1%</t>
+          <t>SWAllied 26.7%, Laboratory 32.4%, MS 26.7%, Depreciation 14.1%</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1794,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MS 69.4%, GS 30.6%</t>
+          <t>MS 35.7%, GS 64.3%</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1806,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SWDoc 70.9%, Laboratory 9.1%, MS 20.0%</t>
+          <t>Laboratory 19.5%, MS 80.5%</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1815,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2242,7 +2770,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2313,7 +2841,7 @@
         <v>5898.341</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>7398.514</v>
+        <v>7398.503</v>
       </c>
     </row>
     <row r="5">
@@ -2378,7 +2906,7 @@
         <v>8670.219999999999</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>27548.855</v>
+        <v>27548.844</v>
       </c>
     </row>
     <row r="10">
@@ -2391,7 +2919,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>7855.305</v>
+        <v>7855.316</v>
       </c>
     </row>
     <row r="11">
@@ -2404,7 +2932,7 @@
         <v>0</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7855.305</v>
+        <v>7855.316</v>
       </c>
     </row>
     <row r="12">
@@ -2417,7 +2945,7 @@
         <v>708.082</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>504.73</v>
+        <v>248.983</v>
       </c>
     </row>
     <row r="13">
@@ -2430,7 +2958,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>45.455</v>
+        <v>48.967</v>
       </c>
     </row>
     <row r="14">
@@ -2443,7 +2971,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>60.588</v>
+        <v>47.372</v>
       </c>
     </row>
     <row r="15">
@@ -2456,7 +2984,7 @@
         <v>2316.482</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1142.247</v>
+        <v>321.136</v>
       </c>
     </row>
     <row r="16">
@@ -2469,7 +2997,7 @@
         <v>356.264</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>351.976</v>
+        <v>351.97</v>
       </c>
     </row>
     <row r="17">
@@ -2482,7 +3010,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>106.897</v>
+        <v>106.887</v>
       </c>
     </row>
     <row r="18">
@@ -2495,7 +3023,7 @@
         <v>1064.346</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>7396.432</v>
+        <v>7396.459</v>
       </c>
     </row>
     <row r="19">
@@ -2508,7 +3036,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>94.539</v>
+        <v>93.92400000000001</v>
       </c>
     </row>
     <row r="20">
@@ -2534,7 +3062,7 @@
         <v>1422.734</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>513.547</v>
+        <v>180.972</v>
       </c>
     </row>
     <row r="22">
@@ -2547,7 +3075,7 @@
         <v>14222.342</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>6706.191</v>
+        <v>7991.475</v>
       </c>
     </row>
     <row r="23">
@@ -2573,7 +3101,7 @@
         <v>4872.231</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1103.096</v>
+        <v>1237.553</v>
       </c>
     </row>
     <row r="25">
@@ -2712,7 +3240,7 @@
         <v>11.273</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>20.274</v>
+        <v>9.978</v>
       </c>
     </row>
     <row r="36">
@@ -2725,7 +3253,7 @@
         <v>0</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>1.176</v>
+        <v>1.103</v>
       </c>
     </row>
     <row r="37">
@@ -2738,7 +3266,7 @@
         <v>0</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.324</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="38">
@@ -2751,7 +3279,7 @@
         <v>13.156</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>38.601</v>
+        <v>9.717000000000001</v>
       </c>
     </row>
     <row r="39">
@@ -2803,7 +3331,7 @@
         <v>0</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>3.842</v>
+        <v>3.812</v>
       </c>
     </row>
     <row r="43">
@@ -2816,7 +3344,7 @@
         <v>16.294</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>20.162</v>
+        <v>6.302</v>
       </c>
     </row>
     <row r="44">
@@ -2829,7 +3357,7 @@
         <v>169.098</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>212.443</v>
+        <v>253.06</v>
       </c>
     </row>
     <row r="45">
@@ -2855,7 +3383,7 @@
         <v>57.621</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>36.24</v>
+        <v>49.03</v>
       </c>
     </row>
     <row r="47">
@@ -2876,7 +3404,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2975,49 +3503,49 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: fils residuals {SWNurs:-45, SWDoc:-10, SWAllied:+33, Laboratory:-22, Pharmacy:+17, MS:-20, GS:-17, Depreciation:-25, OHF:-12, OHDepreciation:+60, OHC:+41} absorbed by claim 1740MF4159-d7a251</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: fils residuals {SWNurs:+43, SWDoc:-12, SWAllied:+26, Laboratory:-53, Pharmacy:-50, MS:-29, GS:+17, Depreciation:-42, OHF:+15, OHDepreciation:+50, OHC:+35} absorbed by claim 1740MF4159-d7a251</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Anaesthesia profile SWDoc 81.3%, Pharmacy 5.0%, MS 13.8%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Anaesthesia profile SWNurs 6.6%, SWDoc 85.8%, Pharmacy 4.9%, MS 2.7%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Dental profile SWNurs 6.1%, SWDoc 33.8%, SWAllied 1.7%, Laboratory 0.1%, Pharmacy 0.0%, MS 4.8%, GS 0.3%, Depreciation 1.7%, OHF 48.5%, OHDepreciation 0.7%, OHC 2.3%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Dental profile SWNurs 4.1%, SWDoc 42.1%, SWAllied 0.4%, Laboratory 0.0%, Pharmacy 0.0%, MS 1.1%, GS 0.2%, Depreciation 0.6%, OHF 48.5%, OHDepreciation 0.7%, OHC 2.3%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Imaging profile SWNurs 21.7%, SWAllied 30.6%, MS 16.9%, Depreciation 30.7%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Imaging profile SWNurs 63.6%, SWAllied 11.5%, MS 6.9%, Depreciation 18.1%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Laboratory profile SWDoc 42.7%, SWAllied 8.7%, Laboratory 36.5%, MS 12.1%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Laboratory profile SWAllied 26.7%, Laboratory 32.4%, MS 26.7%, Depreciation 14.1%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket OP profile MS 69.4%, GS 30.6%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket OP profile MS 35.7%, GS 64.3%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Prosthesis profile SWDoc 70.9%, Laboratory 9.1%, MS 20.0%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Prosthesis profile Laboratory 19.5%, MS 80.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Month report: replace the bucket-profile sheet with two explicit sheets (where each cost type goes; what each bucket is made of)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/output/January_Model_Report.xlsx
+++ b/output/January_Model_Report.xlsx
@@ -10,11 +10,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost types" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buckets" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Type x Bucket" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bucket profiles" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implant claims" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim examples" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Where each cost type goes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What each bucket is made of" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Type x Bucket" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implant claims" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim examples" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1194,6 +1195,1174 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Cost type</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Month total AED</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Anaesthesia AED</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Dental AED</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Imaging AED</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Laboratory AED</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Prosthesis AED</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Anaesthesia %</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Dental %</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Imaging %</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Laboratory %</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Prosthesis %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SWNurs</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>25100</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>251</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>23845</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>1004</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SWDoc</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>171870</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>3437.4</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>168432.6</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SWAllied</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>14150</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>7150</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.4946996466431096</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0.5053003533568905</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>17278.94</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>17278.94</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>1252</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>1252</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Prostheses</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>52796</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>52796</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>31662.75</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>31662.75</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Depreciation</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>10556.61</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>10134.346</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>422.264</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.9600000378909518</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0.03999996210904827</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>174794.2</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>174794.2</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OHDepreciation</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OHC</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>8317</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>8317</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Read a row: e.g. SWDoc = the dentists' pay for the month and the share of it sitting in each bucket (98% Dental, 2% Anaesthesia by ruling).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="15" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
+    <col width="15" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Bucket</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Bucket total AED</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>SWNurs AED</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>SWDoc AED</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>SWAllied AED</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Laboratory AED</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Pharmacy AED</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Prostheses AED</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>MS AED</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>GS AED</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Depreciation AED</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>OHF AED</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>OHDepreciation AED</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>OHC AED</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>SWNurs %</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>SWDoc %</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>SWAllied %</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>Laboratory %</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>Pharmacy %</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>Prostheses %</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
+        <is>
+          <t>MS %</t>
+        </is>
+      </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>GS %</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Depreciation %</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>OHF %</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>OHDepreciation %</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>OHC %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Anaesthesia</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>4940.4</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>251</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>3437.4</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>1252</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>0.05080560278519958</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>0.6957736215691038</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.2534207756456967</v>
+      </c>
+      <c r="T2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dental</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>427710.696</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>23845</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>168432.6</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>31662.75</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>10134.346</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>174794.2</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="N3" s="7" t="n">
+        <v>8317</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0.05575030089965297</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>0.3938002990694439</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>0.01636620282229276</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <v>0.07402842691593572</v>
+      </c>
+      <c r="V3" s="4" t="n">
+        <v>0.002338028974613251</v>
+      </c>
+      <c r="W3" s="4" t="n">
+        <v>0.0236943945867559</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>0.4086739041943436</v>
+      </c>
+      <c r="Y3" s="4" t="n">
+        <v>0.005903055555103537</v>
+      </c>
+      <c r="Z3" s="4" t="n">
+        <v>0.01944538698185841</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Imaging</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>1426.264</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>1004</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>422.264</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0.7039369990408507</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="4" t="n">
+        <v>0.2960630009591492</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>24428.94</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>7150</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>17278.94</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>0.2926856425207152</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>0.7073143574792848</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Prosthesis</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>52796</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>52796</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Read a row: e.g. Anaesthesia = a small bucket (drugs + 2% of dentists + 1% of nurses); its % columns describe that bucket only, not the salaries.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1668,97 +2837,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="150" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Bucket</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Cost-type profile fitted for the month (share of the bucket)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Anaesthesia</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>SWNurs 5.1%, SWDoc 69.6%, Pharmacy 25.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SWNurs 70.4%, Depreciation 29.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Dental</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SWNurs 5.6%, SWDoc 39.4%, SWAllied 1.6%, MS 7.4%, GS 0.2%, Depreciation 2.4%, OHF 40.9%, OHDepreciation 0.6%, OHC 1.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Laboratory</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SWAllied 29.3%, Laboratory 70.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Prosthesis</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Prostheses 100.0%</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2713,7 +3792,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3360,7 +4439,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
January report: add the cost-type x bucket tuning grid (percent of each cost type per bucket)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/output/January_Model_Report.xlsx
+++ b/output/January_Model_Report.xlsx
@@ -8,14 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost types" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buckets" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Where each cost type goes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What each bucket is made of" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Type x Bucket" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implant claims" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim examples" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning grid" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost types" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buckets" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Where each cost type goes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What each bucket is made of" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Type x Bucket" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implant claims" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim examples" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -65,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -75,6 +76,9 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -480,10 +484,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr"/>
       <c r="B5" s="1" t="inlineStr">
@@ -580,7 +581,6 @@
           <t>Claims with implant codes</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
         <v>23</v>
       </c>
@@ -617,10 +617,152 @@
           <t>Claim set and identity fields</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>unchanged</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="160" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: claim totals +0.068 AED vs ledger absorbed by claim 1740MF4159-d7a251</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: implant pools from stock bone_graft 13,985.00, fixtures 31,199.00, abutments 7,612.00; coded claims in activity: 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bone_graft pool 13,985.000 AED placed on 8 claims by units (26 units; 537.885 AED per unit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: fixtures pool 31,199.000 AED placed on 7 claims by units (13 units; 2,399.923 AED per unit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2209MF4159-fa59f1 share 422.889 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2180MF4159-2f6011 share 422.889 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2224MF4159-3c483f share 422.889 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2156MF4159-53564a share 422.889 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2210MF4159-e60915 share 422.889 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2243MF4159-37c990 share 845.777 capped at its Dental amount 530.367</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2252MF4159-582382 share 422.889 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments pool 7,612.000 AED placed on 11 claims by units (18 units; 422.889 AED per unit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: fils residuals {SWDoc:-46, SWAllied:-1, Laboratory:-50, Pharmacy:-7, MS:-9, GS:+44, Depreciation:-15, OHF:+44, OHDepreciation:+42, OHC:-2} absorbed by claim index 307</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Anaesthesia profile SWNurs 5.1%, SWDoc 69.6%, Pharmacy 25.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Imaging profile SWNurs 70.4%, Depreciation 29.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Dental profile SWNurs 5.6%, SWDoc 39.4%, SWAllied 1.6%, MS 7.4%, GS 0.2%, Depreciation 2.4%, OHF 40.9%, OHDepreciation 0.6%, OHC 1.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Laboratory profile SWAllied 29.3%, Laboratory 70.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Prosthesis profile Prostheses 100.0%</t>
         </is>
       </c>
     </row>
@@ -630,6 +772,1121 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Cost type</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>January AED</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Allied</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Anaesthesia</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Dental</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>ICU</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>Imaging</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>Physician</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="M1" s="9" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="N1" s="9" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="O1" s="9" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="P1" s="9" t="inlineStr">
+        <is>
+          <t>Prosthesis</t>
+        </is>
+      </c>
+      <c r="Q1" s="9" t="inlineStr">
+        <is>
+          <t>SPS</t>
+        </is>
+      </c>
+      <c r="R1" s="9" t="inlineStr">
+        <is>
+          <t>Ward</t>
+        </is>
+      </c>
+      <c r="S1" s="9" t="inlineStr">
+        <is>
+          <t>Row total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SWNurs</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>25100</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SWDoc</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>171870</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SWAllied</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>14150</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0.4946996466431096</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0.5053003533568905</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SWNonClin</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>17278.94</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Imaging</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>1252</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Prostheses</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>52796</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>31662.75</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Depreciation</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>10556.61</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0.9600000378909518</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.03999996210904827</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>174794.2</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OHDepreciation</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OHC</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>8317</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NABMs</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Each row = one DOH cost type (Standard v2.1 Appendix 1); each column = one DOH cost bucket (Appendix 2). Cells = share of that cost type placed in that bucket, January 2025. Rows sum to 100%. Rows with 0 AED have no January amount in the ledger.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -986,7 +2243,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1189,7 +2446,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1766,7 +3023,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2357,7 +3614,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2837,7 +4094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2943,7 +4200,6 @@
       <c r="J2" s="2" t="n">
         <v>17466.175</v>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2980,7 +4236,6 @@
       <c r="J3" s="2" t="n">
         <v>8453.815000000001</v>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3017,7 +4272,6 @@
       <c r="J4" s="2" t="n">
         <v>3621.915</v>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3054,7 +4308,6 @@
       <c r="J5" s="2" t="n">
         <v>4701.498</v>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3091,7 +4344,6 @@
       <c r="J6" s="2" t="n">
         <v>3191.07</v>
       </c>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3128,7 +4380,6 @@
       <c r="J7" s="2" t="n">
         <v>3761.839</v>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3165,7 +4416,6 @@
       <c r="J8" s="2" t="n">
         <v>1989.799</v>
       </c>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3202,7 +4452,6 @@
       <c r="J9" s="2" t="n">
         <v>3594.324</v>
       </c>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3239,7 +4488,6 @@
       <c r="J10" s="2" t="n">
         <v>920.035</v>
       </c>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3276,7 +4524,6 @@
       <c r="J11" s="2" t="n">
         <v>541.308</v>
       </c>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3313,7 +4560,6 @@
       <c r="J12" s="2" t="n">
         <v>541.308</v>
       </c>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3350,7 +4596,6 @@
       <c r="J13" s="2" t="n">
         <v>2002.748</v>
       </c>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3674,7 +4919,6 @@
       <c r="J21" s="2" t="n">
         <v>622.299</v>
       </c>
-      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3711,7 +4955,6 @@
       <c r="J22" s="2" t="n">
         <v>229.03</v>
       </c>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3748,7 +4991,6 @@
       <c r="J23" s="2" t="n">
         <v>3713.447</v>
       </c>
-      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3785,14 +5027,13 @@
       <c r="J24" s="2" t="n">
         <v>3739.535</v>
       </c>
-      <c r="K24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4139,7 +5380,6 @@
         <v>35404.16</v>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
@@ -4432,149 +5672,6 @@
       </c>
       <c r="C48" s="2" t="n">
         <v>563.658</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="160" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: claim totals +0.068 AED vs ledger absorbed by claim 1740MF4159-d7a251</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: implant pools from stock bone_graft 13,985.00, fixtures 31,199.00, abutments 7,612.00; coded claims in activity: 19</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bone_graft pool 13,985.000 AED placed on 8 claims by units (26 units; 537.885 AED per unit)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: fixtures pool 31,199.000 AED placed on 7 claims by units (13 units; 2,399.923 AED per unit)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2209MF4159-fa59f1 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2180MF4159-2f6011 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2224MF4159-3c483f share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2156MF4159-53564a share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2210MF4159-e60915 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2243MF4159-37c990 share 845.777 capped at its Dental amount 530.367</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2252MF4159-582382 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments pool 7,612.000 AED placed on 11 claims by units (18 units; 422.889 AED per unit)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: fils residuals {SWDoc:-46, SWAllied:-1, Laboratory:-50, Pharmacy:-7, MS:-9, GS:+44, Depreciation:-15, OHF:+44, OHDepreciation:+42, OHC:-2} absorbed by claim index 307</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Anaesthesia profile SWNurs 5.1%, SWDoc 69.6%, Pharmacy 25.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Imaging profile SWNurs 70.4%, Depreciation 29.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Dental profile SWNurs 5.6%, SWDoc 39.4%, SWAllied 1.6%, MS 7.4%, GS 0.2%, Depreciation 2.4%, OHF 40.9%, OHDepreciation 0.6%, OHC 1.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Laboratory profile SWAllied 29.3%, Laboratory 70.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Prosthesis profile Prostheses 100.0%</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct implant code pools from the revised LAB/Prosthesis/Implants list; re-run January; record prostheses classification guidance
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/output/January_Model_Report.xlsx
+++ b/output/January_Model_Report.xlsx
@@ -8,15 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning grid" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost types" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buckets" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Where each cost type goes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What each bucket is made of" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Type x Bucket" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implant claims" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim examples" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost types" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buckets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Where each cost type goes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What each bucket is made of" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Type x Bucket" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implant claims" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim examples" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -66,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -76,9 +75,6 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -484,7 +480,10 @@
         <v>831</v>
       </c>
     </row>
-    <row r="4"/>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+    </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr"/>
       <c r="B5" s="1" t="inlineStr">
@@ -581,8 +580,9 @@
           <t>Claims with implant codes</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
@@ -595,7 +595,7 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13">
@@ -617,152 +617,10 @@
           <t>Claim set and identity fields</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>unchanged</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="160" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: claim totals +0.068 AED vs ledger absorbed by claim 1740MF4159-d7a251</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: implant pools from stock bone_graft 13,985.00, fixtures 31,199.00, abutments 7,612.00; coded claims in activity: 19</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bone_graft pool 13,985.000 AED placed on 8 claims by units (26 units; 537.885 AED per unit)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: fixtures pool 31,199.000 AED placed on 7 claims by units (13 units; 2,399.923 AED per unit)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2209MF4159-fa59f1 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2180MF4159-2f6011 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2224MF4159-3c483f share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2156MF4159-53564a share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2210MF4159-e60915 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2243MF4159-37c990 share 845.777 capped at its Dental amount 530.367</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2252MF4159-582382 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments pool 7,612.000 AED placed on 11 claims by units (18 units; 422.889 AED per unit)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: fils residuals {SWDoc:-46, SWAllied:-1, Laboratory:-50, Pharmacy:-7, MS:-9, GS:+44, Depreciation:-15, OHF:+44, OHDepreciation:+42, OHC:-2} absorbed by claim index 307</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Anaesthesia profile SWNurs 5.1%, SWDoc 69.6%, Pharmacy 25.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Imaging profile SWNurs 70.4%, Depreciation 29.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Dental profile SWNurs 5.6%, SWDoc 39.4%, SWAllied 1.6%, MS 7.4%, GS 0.2%, Depreciation 2.4%, OHF 40.9%, OHDepreciation 0.6%, OHC 1.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Laboratory profile SWAllied 29.3%, Laboratory 70.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Prosthesis profile Prostheses 100.0%</t>
         </is>
       </c>
     </row>
@@ -772,1121 +630,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:S19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>Cost type</t>
-        </is>
-      </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>January AED</t>
-        </is>
-      </c>
-      <c r="C1" s="9" t="inlineStr">
-        <is>
-          <t>Allied</t>
-        </is>
-      </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Anaesthesia</t>
-        </is>
-      </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>Dental</t>
-        </is>
-      </c>
-      <c r="F1" s="9" t="inlineStr">
-        <is>
-          <t>ED</t>
-        </is>
-      </c>
-      <c r="G1" s="9" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="H1" s="9" t="inlineStr">
-        <is>
-          <t>ICU</t>
-        </is>
-      </c>
-      <c r="I1" s="9" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="J1" s="9" t="inlineStr">
-        <is>
-          <t>Laboratory</t>
-        </is>
-      </c>
-      <c r="K1" s="9" t="inlineStr">
-        <is>
-          <t>Physician</t>
-        </is>
-      </c>
-      <c r="L1" s="9" t="inlineStr">
-        <is>
-          <t>OP</t>
-        </is>
-      </c>
-      <c r="M1" s="9" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="N1" s="9" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="O1" s="9" t="inlineStr">
-        <is>
-          <t>Pharmacy</t>
-        </is>
-      </c>
-      <c r="P1" s="9" t="inlineStr">
-        <is>
-          <t>Prosthesis</t>
-        </is>
-      </c>
-      <c r="Q1" s="9" t="inlineStr">
-        <is>
-          <t>SPS</t>
-        </is>
-      </c>
-      <c r="R1" s="9" t="inlineStr">
-        <is>
-          <t>Ward</t>
-        </is>
-      </c>
-      <c r="S1" s="9" t="inlineStr">
-        <is>
-          <t>Row total</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SWNurs</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="n">
-        <v>25100</v>
-      </c>
-      <c r="C2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="J2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>SWDoc</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="n">
-        <v>171870</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>SWAllied</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>14150</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>0.4946996466431096</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>0.5053003533568905</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SWNonClin</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Laboratory</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>17278.94</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Pharmacy</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>1252</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Prostheses</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>52796</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>31662.75</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Hotel</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Depreciation</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>10556.61</v>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>0.9600000378909518</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>0.03999996210904827</v>
-      </c>
-      <c r="J13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>OHF</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>174794.2</v>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>OHDepreciation</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>2524.8</v>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>OHC</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n">
-        <v>8317</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>NABMs</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Each row = one DOH cost type (Standard v2.1 Appendix 1); each column = one DOH cost bucket (Appendix 2). Cells = share of that cost type placed in that bucket, January 2025. Rows sum to 100%. Rows with 0 AED have no January amount in the ledger.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2243,7 +986,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2300,13 +1043,13 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>4940.413</v>
+        <v>4940.42</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>4940.413</v>
+        <v>4940.42</v>
       </c>
     </row>
     <row r="3">
@@ -2322,13 +1065,13 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>242074.682</v>
+        <v>242074.669</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>185636</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>427710.682</v>
+        <v>427710.669</v>
       </c>
     </row>
     <row r="4">
@@ -2344,13 +1087,13 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1426.248</v>
+        <v>1426.243</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1426.248</v>
+        <v>1426.243</v>
       </c>
     </row>
     <row r="5">
@@ -2366,13 +1109,13 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>24428.957</v>
+        <v>24428.968</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>24428.957</v>
+        <v>24428.968</v>
       </c>
     </row>
     <row r="6">
@@ -2446,7 +1189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3023,7 +1766,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3614,7 +2357,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4094,13 +2837,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4189,17 +2932,18 @@
         <v>35404.16</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>17378.462</v>
+        <v>17179.245</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>17378.462</v>
+        <v>17179.245</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>32632.213</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>17466.175</v>
-      </c>
+        <v>17659.218</v>
+      </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4225,17 +2969,18 @@
         <v>19146.779</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>10427.077</v>
+        <v>10307.547</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10427.077</v>
+        <v>10307.547</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>17735.28</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>8453.815000000001</v>
-      </c>
+        <v>8569.722</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4261,17 +3006,18 @@
         <v>7216.203</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>3475.692</v>
+        <v>3435.849</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>3475.692</v>
+        <v>3435.849</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>6648.202</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>3621.915</v>
-      </c>
+        <v>3660.503</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4297,17 +3043,18 @@
         <v>8333.188</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>3475.692</v>
+        <v>3435.849</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>3475.692</v>
+        <v>3435.849</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>7605.273</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>4701.498</v>
-      </c>
+        <v>4740.073</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4333,17 +3080,18 @@
         <v>6771.552</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>3475.692</v>
+        <v>3435.849</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>3475.692</v>
+        <v>3435.849</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>6243.998</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>3191.07</v>
-      </c>
+        <v>3229.653</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4369,233 +3117,240 @@
         <v>7360.849</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>3475.692</v>
+        <v>3435.849</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>3475.692</v>
+        <v>3435.849</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>6774.365</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>3761.839</v>
-      </c>
+        <v>3800.427</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2158MF4159-2e9a64</t>
+          <t>1430MF4159-33eb6a</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>67115, 67115, 67115, 67115, 67115, 67115</t>
+          <t>42211, 42702, 79933</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>5421.528</v>
+        <v>6654.841</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>3166.769</v>
+        <v>2917.886</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>3166.769</v>
+        <v>2917.886</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>3667.782</v>
+        <v>6122.045</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>1989.799</v>
-      </c>
+        <v>3613.593</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1430MF4159-33eb6a</t>
+          <t>2158MF4159-2e9a64</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>42211, 42702, 79933</t>
+          <t>67115, 67115, 67115, 67115, 67115, 67115</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>6654.841</v>
+        <v>5421.528</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>2937.808</v>
+        <v>1709.948</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>2937.808</v>
+        <v>1709.948</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>6122.045</v>
+        <v>3667.782</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>3594.324</v>
-      </c>
+        <v>3275.367</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1938MF4159-4ad9ae</t>
+          <t>1652MF4159-851edd</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>67155, 67155</t>
+          <t>67205, 67205, 67205, 67205, 67205</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>2177.718</v>
+        <v>13052.917</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>1136.454</v>
+        <v>1467.049</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1136.454</v>
+        <v>1467.049</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>1465.633</v>
+        <v>8964.673000000001</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>920.035</v>
-      </c>
+        <v>10234.983</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1653MF4159-47fd9e</t>
+          <t>1651MF4159-7d496b</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>27205</t>
+          <t>67205, 67205</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>1205.379</v>
+        <v>5892.965</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>593.6559999999999</v>
+        <v>590.131</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>593.6559999999999</v>
+        <v>590.131</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>821.533</v>
+        <v>4054.36</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>541.308</v>
-      </c>
+        <v>4680.766</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1683MF4159-389500</t>
+          <t>1936MF4159-12a7bc</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>27205</t>
+          <t>67205, 67205</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>1205.379</v>
+        <v>3562.565</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>593.6559999999999</v>
+        <v>578.639</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>593.6559999999999</v>
+        <v>578.639</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>821.533</v>
+        <v>2424.419</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>541.308</v>
-      </c>
+        <v>2635.571</v>
+      </c>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2616MF4159-6c718c</t>
+          <t>1938MF4159-4ad9ae</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>42631</t>
+          <t>67155, 67155</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>2639.589</v>
+        <v>2177.718</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>537.885</v>
+        <v>571.8099999999999</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>537.885</v>
+        <v>571.8099999999999</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>2246.368</v>
+        <v>1465.633</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>2002.748</v>
-      </c>
+        <v>1418.915</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4634,101 +3389,93 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>claim 2243MF4159-37c990 share 845.777 capped at its Dental amount 530.367</t>
+          <t>claim 2243MF4159-37c990 share 563.852 capped at its Dental amount 530.367</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2156MF4159-53564a</t>
+          <t>2074MF4159-800bec</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>27155</t>
+          <t>79356</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
         <v>1</v>
       </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
       <c r="F15" s="2" t="n">
-        <v>265.183</v>
+        <v>5675.997</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>265.183</v>
+        <v>517.963</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>265.183</v>
+        <v>517.963</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>206.842</v>
+        <v>5017.485</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>claim 2156MF4159-53564a share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
+        <v>4973.663</v>
+      </c>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2180MF4159-2f6011</t>
+          <t>2616MF4159-6c718c</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>27155</t>
+          <t>42631</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
         <v>1</v>
       </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
       <c r="F16" s="2" t="n">
-        <v>265.183</v>
+        <v>2639.589</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>265.183</v>
+        <v>517.963</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>265.183</v>
+        <v>517.963</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>206.842</v>
+        <v>2246.368</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>claim 2180MF4159-2f6011 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
+        <v>2021.731</v>
+      </c>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2209MF4159-fa59f1</t>
+          <t>1653MF4159-47fd9e</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>27155</t>
+          <t>27205</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -4741,35 +3488,31 @@
         <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>265.183</v>
+        <v>1205.379</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>265.183</v>
+        <v>286.479</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>265.183</v>
+        <v>286.479</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>206.842</v>
+        <v>821.533</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>claim 2209MF4159-fa59f1 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
+        <v>813.111</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2210MF4159-e60915</t>
+          <t>1683MF4159-389500</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>27155</t>
+          <t>27205</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -4782,30 +3525,26 @@
         <v>0</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>265.183</v>
+        <v>1205.379</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>265.183</v>
+        <v>286.479</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>265.183</v>
+        <v>286.479</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>206.842</v>
+        <v>821.533</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>claim 2210MF4159-e60915 share 422.889 capped at its Dental amount 265.183</t>
-        </is>
-      </c>
+        <v>813.111</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2224MF4159-3c483f</t>
+          <t>2156MF4159-53564a</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4839,14 +3578,14 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>claim 2224MF4159-3c483f share 422.889 capped at its Dental amount 265.183</t>
+          <t>claim 2156MF4159-53564a share 281.926 capped at its Dental amount 265.183</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2252MF4159-582382</t>
+          <t>2180MF4159-2f6011</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4880,160 +3619,254 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>claim 2252MF4159-582382 share 422.889 capped at its Dental amount 265.183</t>
+          <t>claim 2180MF4159-2f6011 share 281.926 capped at its Dental amount 265.183</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2028MF4159-507c9c</t>
+          <t>2209MF4159-fa59f1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>29311</t>
+          <t>27155</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>675.0119999999999</v>
+        <v>265.183</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0</v>
+        <v>265.183</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>0</v>
+        <v>265.183</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>540.143</v>
+        <v>206.842</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>622.299</v>
+        <v>0</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>claim 2209MF4159-fa59f1 share 281.926 capped at its Dental amount 265.183</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2054MF4159-8bdf8c</t>
+          <t>2210MF4159-e60915</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>29311, 29311</t>
+          <t>27155</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>235.719</v>
+        <v>265.183</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0</v>
+        <v>265.183</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>0</v>
+        <v>265.183</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>213.326</v>
+        <v>206.842</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>229.03</v>
+        <v>0</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>claim 2210MF4159-e60915 share 281.926 capped at its Dental amount 265.183</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2141MF4159-bd9d96</t>
+          <t>2224MF4159-3c483f</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>73111</t>
+          <t>27155</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>3857.213</v>
+        <v>265.183</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0</v>
+        <v>265.183</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0</v>
+        <v>265.183</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>3400.589</v>
+        <v>206.842</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>3713.447</v>
+        <v>0</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>claim 2224MF4159-3c483f share 281.926 capped at its Dental amount 265.183</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2225MF4159-e8bd9a</t>
+          <t>2252MF4159-582382</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>73111</t>
+          <t>27155</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>3874.433</v>
+        <v>265.183</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0</v>
+        <v>265.183</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0</v>
+        <v>265.183</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>3469.881</v>
+        <v>206.842</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>3739.535</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>claim 2252MF4159-582382 share 281.926 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2028MF4159-507c9c</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>29311</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>675.0119999999999</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>540.143</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>622.294</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2054MF4159-8bdf8c</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>29311, 29311</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>235.719</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>213.326</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>229.031</v>
+      </c>
+      <c r="K26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5091,7 +3924,7 @@
         <v>1826.525</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>230.518</v>
+        <v>233.056</v>
       </c>
     </row>
     <row r="4">
@@ -5104,7 +3937,7 @@
         <v>5898.341</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>10996.837</v>
+        <v>11118.489</v>
       </c>
     </row>
     <row r="5">
@@ -5117,7 +3950,7 @@
         <v>783.068</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>60.66</v>
+        <v>61.342</v>
       </c>
     </row>
     <row r="6">
@@ -5130,7 +3963,7 @@
         <v>132.745</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>268.345</v>
+        <v>271.299</v>
       </c>
     </row>
     <row r="7">
@@ -5156,7 +3989,7 @@
         <v>11.862</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>17378.462</v>
+        <v>17179.245</v>
       </c>
     </row>
     <row r="9">
@@ -5169,7 +4002,7 @@
         <v>8670.219999999999</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>28934.822</v>
+        <v>28863.431</v>
       </c>
     </row>
     <row r="10">
@@ -5182,7 +4015,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>6469.338</v>
+        <v>6540.729</v>
       </c>
     </row>
     <row r="11">
@@ -5195,7 +4028,7 @@
         <v>0</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>6469.338</v>
+        <v>6540.729</v>
       </c>
     </row>
     <row r="12">
@@ -5208,7 +4041,7 @@
         <v>708.082</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>365.052</v>
+        <v>369.097</v>
       </c>
     </row>
     <row r="13">
@@ -5221,7 +4054,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>38.044</v>
+        <v>38.501</v>
       </c>
     </row>
     <row r="14">
@@ -5234,7 +4067,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>38.509</v>
+        <v>38.972</v>
       </c>
     </row>
     <row r="15">
@@ -5247,7 +4080,7 @@
         <v>2316.482</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1075.462</v>
+        <v>1087.102</v>
       </c>
     </row>
     <row r="16">
@@ -5260,7 +4093,7 @@
         <v>356.264</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>273.587</v>
+        <v>276.65</v>
       </c>
     </row>
     <row r="17">
@@ -5273,7 +4106,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>89.68899999999999</v>
+        <v>90.682</v>
       </c>
     </row>
     <row r="18">
@@ -5286,7 +4119,7 @@
         <v>1064.346</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>6106.062</v>
+        <v>6173.397</v>
       </c>
     </row>
     <row r="19">
@@ -5299,7 +4132,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>51.371</v>
+        <v>51.924</v>
       </c>
     </row>
     <row r="20">
@@ -5312,7 +4145,7 @@
         <v>0</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>17378.462</v>
+        <v>17179.245</v>
       </c>
     </row>
     <row r="21">
@@ -5325,7 +4158,7 @@
         <v>1422.734</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>454.851</v>
+        <v>459.78</v>
       </c>
     </row>
     <row r="22">
@@ -5338,7 +4171,7 @@
         <v>14222.342</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>8381.635</v>
+        <v>8474.352999999999</v>
       </c>
     </row>
     <row r="23">
@@ -5364,7 +4197,7 @@
         <v>4872.231</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1151.436</v>
+        <v>1164.457</v>
       </c>
     </row>
     <row r="25">
@@ -5380,6 +4213,7 @@
         <v>35404.16</v>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
@@ -5424,7 +4258,7 @@
         <v>75.13500000000001</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>9.169</v>
+        <v>9.166</v>
       </c>
     </row>
     <row r="30">
@@ -5437,7 +4271,7 @@
         <v>128.363</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>325.877</v>
+        <v>325.878</v>
       </c>
     </row>
     <row r="31">
@@ -5450,7 +4284,7 @@
         <v>40.734</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>2.034</v>
+        <v>2.035</v>
       </c>
     </row>
     <row r="32">
@@ -5476,7 +4310,7 @@
         <v>244.232</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>343.236</v>
+        <v>343.235</v>
       </c>
     </row>
     <row r="34">
@@ -5489,7 +4323,7 @@
         <v>0</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>220.422</v>
+        <v>220.423</v>
       </c>
     </row>
     <row r="35">
@@ -5502,7 +4336,7 @@
         <v>0</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>220.422</v>
+        <v>220.423</v>
       </c>
     </row>
     <row r="36">
@@ -5515,7 +4349,7 @@
         <v>11.273</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>18.145</v>
+        <v>18.142</v>
       </c>
     </row>
     <row r="37">
@@ -5528,7 +4362,7 @@
         <v>0</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>1.074</v>
+        <v>1.076</v>
       </c>
     </row>
     <row r="38">
@@ -5554,7 +4388,7 @@
         <v>13.156</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>38.314</v>
+        <v>38.306</v>
       </c>
     </row>
     <row r="40">
@@ -5593,7 +4427,7 @@
         <v>17.537</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>207.688</v>
+        <v>207.689</v>
       </c>
     </row>
     <row r="43">
@@ -5606,7 +4440,7 @@
         <v>0</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>4.097</v>
+        <v>4.094</v>
       </c>
     </row>
     <row r="44">
@@ -5619,7 +4453,7 @@
         <v>16.294</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>11.079</v>
+        <v>11.078</v>
       </c>
     </row>
     <row r="45">
@@ -5632,7 +4466,7 @@
         <v>169.098</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>237.255</v>
+        <v>237.257</v>
       </c>
     </row>
     <row r="46">
@@ -5658,7 +4492,7 @@
         <v>57.621</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>32.714</v>
+        <v>32.724</v>
       </c>
     </row>
     <row r="48">
@@ -5672,6 +4506,149 @@
       </c>
       <c r="C48" s="2" t="n">
         <v>563.658</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="160" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: claim totals +0.068 AED vs ledger absorbed by claim 1740MF4159-d7a251</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: implant pools from stock bone_graft 13,985.00, fixtures 31,199.00, abutments 7,612.00; coded claims in activity: 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bone_graft pool 13,985.000 AED placed on 9 claims by units (27 units; 517.963 AED per unit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: fixtures pool 31,199.000 AED placed on 7 claims by units (13 units; 2,399.923 AED per unit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2209MF4159-fa59f1 share 281.926 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2180MF4159-2f6011 share 281.926 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2224MF4159-3c483f share 281.926 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2156MF4159-53564a share 281.926 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2210MF4159-e60915 share 281.926 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2243MF4159-37c990 share 563.852 capped at its Dental amount 530.367</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments: claim 2252MF4159-582382 share 281.926 capped at its Dental amount 265.183</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: abutments pool 7,612.000 AED placed on 14 claims by units (27 units; 281.926 AED per unit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: fils residuals {SWNurs:-28, SWDoc:+31, SWAllied:-38, Laboratory:-22, Pharmacy:+17, MS:-18, GS:-5, Depreciation:+41, OHF:-62, OHDepreciation:+45, OHC:+39} absorbed by claim index 307</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Anaesthesia profile SWNurs 5.1%, SWDoc 69.6%, Pharmacy 25.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Imaging profile SWNurs 70.4%, Depreciation 29.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Dental profile SWNurs 5.6%, SWDoc 39.4%, SWAllied 1.6%, MS 7.4%, GS 0.2%, Depreciation 2.4%, OHF 40.9%, OHDepreciation 0.6%, OHC 1.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Laboratory profile SWAllied 29.3%, Laboratory 70.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Prosthesis profile Prostheses 100.0%</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final tuning grid: rebuild and verify all twelve months, regenerate the month reports
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/output/January_Model_Report.xlsx
+++ b/output/January_Model_Report.xlsx
@@ -1032,13 +1032,13 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>18849.353</v>
+        <v>10653.92</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>18849.353</v>
+        <v>10653.92</v>
       </c>
     </row>
     <row r="3">
@@ -1054,13 +1054,13 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>234175.887</v>
+        <v>231860.049</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>130158.78</v>
+        <v>133926.628</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>364334.667</v>
+        <v>365786.677</v>
       </c>
     </row>
     <row r="4">
@@ -1076,13 +1076,13 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>18619.637</v>
+        <v>15115.9</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6279.8</v>
+        <v>2511.952</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>24899.437</v>
+        <v>17627.852</v>
       </c>
     </row>
     <row r="5">
@@ -1142,13 +1142,13 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>103218.843</v>
+        <v>117233.851</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>103218.843</v>
+        <v>117233.851</v>
       </c>
     </row>
     <row r="8">
@@ -1292,13 +1292,13 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>202921.409</v>
+        <v>202921.41</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>10146.07</v>
+        <v>6087.642</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>152191.057</v>
+        <v>156249.486</v>
       </c>
       <c r="E3" s="7" t="n">
         <v>10146.07</v>
@@ -1307,16 +1307,16 @@
         <v>30438.212</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.04999999778239269</v>
+        <v>0.02999999852159513</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.7500000012320042</v>
+        <v>0.7700000014784049</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>0.04999999778239269</v>
+        <v>0.04999999753599189</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.1500000032032106</v>
+        <v>0.1500000024640081</v>
       </c>
     </row>
     <row r="4">
@@ -1397,28 +1397,28 @@
         <v>70074.94</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>3503.747</v>
+        <v>0</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>7007.494</v>
+        <v>0</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>3503.747</v>
+        <v>0</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>56059.952</v>
+        <v>70074.94</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.09999999999999999</v>
+        <v>0</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0.7999999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1428,13 +1428,13 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>31662.752</v>
+        <v>31662.751</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1583.138</v>
+        <v>949.883</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>26913.338</v>
+        <v>27546.592</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>1583.138</v>
@@ -1443,16 +1443,16 @@
         <v>1583.138</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.05000001263314067</v>
+        <v>0.03000001484394076</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.8499999621005779</v>
+        <v>0.8699999567314919</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.05000001263314067</v>
+        <v>0.0500000142122837</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.05000001263314067</v>
+        <v>0.0500000142122837</v>
       </c>
     </row>
     <row r="8">
@@ -1536,10 +1536,10 @@
         <v>0</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>119316.941</v>
+        <v>123084.844</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>6279.839</v>
+        <v>2511.936</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>0</v>
@@ -1548,10 +1548,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.9500000000000001</v>
+        <v>0.979999996815205</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>0.05</v>
+        <v>0.02000000318479503</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>0</v>
@@ -1801,13 +1801,13 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>18849.327</v>
+        <v>10653.897</v>
       </c>
       <c r="C2" s="7" t="n">
         <v>1836.541</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>10146.07</v>
+        <v>6087.642</v>
       </c>
       <c r="E2" s="7" t="n">
         <v>0</v>
@@ -1816,10 +1816,10 @@
         <v>1252</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>3503.747</v>
+        <v>0</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>1583.138</v>
+        <v>949.883</v>
       </c>
       <c r="I2" s="7" t="n">
         <v>0</v>
@@ -1837,28 +1837,28 @@
         <v>0</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>0.09743270940124281</v>
+        <v>0.1723820870428915</v>
       </c>
       <c r="O2" s="4" t="n">
-        <v>0.5382722682884116</v>
+        <v>0.5714004931716535</v>
       </c>
       <c r="P2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q2" s="4" t="n">
-        <v>0.0664214695835029</v>
+        <v>0.1175156846363354</v>
       </c>
       <c r="R2" s="4" t="n">
-        <v>0.1858818089367328</v>
+        <v>0</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.08398909945166741</v>
+        <v>0.08915826762732924</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.02800264433844243</v>
+        <v>0.04954346752179039</v>
       </c>
       <c r="V2" s="4" t="n">
         <v>0</v>
@@ -1877,13 +1877,13 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>364334.681</v>
+        <v>365786.773</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>29384.648</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>152191.057</v>
+        <v>156249.486</v>
       </c>
       <c r="E3" s="7" t="n">
         <v>8178.454</v>
@@ -1892,10 +1892,10 @@
         <v>0</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>7007.494</v>
+        <v>0</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>26913.338</v>
+        <v>27546.592</v>
       </c>
       <c r="I3" s="7" t="n">
         <v>1000</v>
@@ -1904,7 +1904,7 @@
         <v>9500.949000000001</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>119316.941</v>
+        <v>123084.844</v>
       </c>
       <c r="L3" s="7" t="n">
         <v>2524.8</v>
@@ -1913,37 +1913,37 @@
         <v>8317</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>0.08065289837175836</v>
+        <v>0.08033272433281781</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>0.4177232224565522</v>
+        <v>0.4271600219945624</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>0.02244764066256981</v>
+        <v>0.02235852852995316</v>
       </c>
       <c r="Q3" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>0.01923367267910463</v>
+        <v>0</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.07386982190696252</v>
+        <v>0.07530778593790213</v>
       </c>
       <c r="T3" s="4" t="n">
-        <v>0.00274472909703592</v>
+        <v>0.002733833133982677</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.02607753116975433</v>
+        <v>0.02597400918047958</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.3274926797320182</v>
+        <v>0.3364934248182889</v>
       </c>
       <c r="W3" s="4" t="n">
-        <v>0.006929892024196292</v>
+        <v>0.006902381896679463</v>
       </c>
       <c r="X3" s="4" t="n">
-        <v>0.02282791190004775</v>
+        <v>0.02273729017533392</v>
       </c>
     </row>
     <row r="4">
@@ -1953,7 +1953,7 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>24899.473</v>
+        <v>17627.823</v>
       </c>
       <c r="C4" s="7" t="n">
         <v>1836.541</v>
@@ -1968,7 +1968,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>3503.747</v>
+        <v>0</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>1583.138</v>
@@ -1980,7 +1980,7 @@
         <v>527.831</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>6279.839</v>
+        <v>2511.936</v>
       </c>
       <c r="L4" s="7" t="n">
         <v>0</v>
@@ -1989,31 +1989,31 @@
         <v>0</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>0.07375822773437815</v>
+        <v>0.1041842205926393</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>0.4074813149659834</v>
+        <v>0.575571356712624</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>0.04105737498942247</v>
+        <v>0.05799394514002098</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>0.1407157091236429</v>
+        <v>0</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.06358118503150649</v>
+        <v>0.08980904788980465</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>0.02119848078712349</v>
+        <v>0.02994306216938983</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2522077073679431</v>
+        <v>0.1424983674955211</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>103218.823</v>
+        <v>117233.811</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>3673.081</v>
@@ -2044,7 +2044,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>56059.952</v>
+        <v>70074.94</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>1583.138</v>
@@ -2065,22 +2065,22 @@
         <v>0</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>0.03558537961627406</v>
+        <v>0.03133124282720793</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>0.2948901287122795</v>
+        <v>0.2596368039251066</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>0.1110692765795246</v>
+        <v>0.09779124215282911</v>
       </c>
       <c r="Q5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>0.5431175280888447</v>
+        <v>0.5977366034786671</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>0.01533768700307695</v>
+        <v>0.01350410761618932</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0</v>
@@ -2206,10 +2206,10 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>10146.07</v>
+        <v>6087.642</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>152191.057</v>
+        <v>156249.486</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>10146.07</v>
@@ -2218,13 +2218,13 @@
         <v>30438.212</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>202921.409</v>
+        <v>202921.41</v>
       </c>
       <c r="G3" s="7" t="n">
         <v>202921.41</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.7500000012320042</v>
+        <v>0.7700000014784049</v>
       </c>
     </row>
     <row r="4">
@@ -2290,16 +2290,16 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>3503.747</v>
+        <v>0</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>7007.494</v>
+        <v>0</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>3503.747</v>
+        <v>0</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>56059.952</v>
+        <v>70074.94</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>70074.94</v>
@@ -2308,7 +2308,7 @@
         <v>70074.94</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.09999999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -2318,10 +2318,10 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>1583.138</v>
+        <v>949.883</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>26913.338</v>
+        <v>27546.592</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>1583.138</v>
@@ -2330,13 +2330,13 @@
         <v>1583.138</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>31662.752</v>
+        <v>31662.751</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>31662.75</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.8499999621005779</v>
+        <v>0.8699999567314919</v>
       </c>
     </row>
     <row r="8">
@@ -2405,10 +2405,10 @@
         <v>0</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>119316.941</v>
+        <v>123084.844</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>6279.839</v>
+        <v>2511.936</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>0</v>
@@ -2420,7 +2420,7 @@
         <v>125596.78</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.9500000000000001</v>
+        <v>0.979999996815205</v>
       </c>
     </row>
     <row r="11">
@@ -2486,16 +2486,16 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>18849.327</v>
+        <v>10653.897</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>364334.681</v>
+        <v>365786.773</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>24899.473</v>
+        <v>17627.823</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>103218.823</v>
+        <v>117233.811</v>
       </c>
       <c r="F13" s="8" t="n">
         <v>511302.304</v>
@@ -2623,13 +2623,13 @@
         <v>18233.212</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>16807.94</v>
+        <v>20454.582</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>32632.213</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>15310.8</v>
+        <v>13806.418</v>
       </c>
       <c r="L2" t="inlineStr"/>
     </row>
@@ -2663,13 +2663,13 @@
         <v>10934.843</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>9875.009</v>
+        <v>12061.978</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>17735.28</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>7486.723</v>
+        <v>6544.666</v>
       </c>
       <c r="L3" t="inlineStr"/>
     </row>
@@ -2703,13 +2703,13 @@
         <v>3649.647</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>3485.077</v>
+        <v>4215.007</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>7605.273</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>4081.493</v>
+        <v>3804.244</v>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
@@ -2743,13 +2743,13 @@
         <v>3647.304</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>3387.721</v>
+        <v>4117.182</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>6774.365</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>3292.392</v>
+        <v>2996.875</v>
       </c>
       <c r="L5" t="inlineStr"/>
     </row>
@@ -2783,13 +2783,13 @@
         <v>3646.956</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>3373.406</v>
+        <v>4102.797</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>6648.202</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>3174.818</v>
+        <v>2876.6</v>
       </c>
       <c r="L6" t="inlineStr"/>
     </row>
@@ -2823,13 +2823,13 @@
         <v>3645.885</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>3328.236</v>
+        <v>4057.413</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>6243.998</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>2814.981</v>
+        <v>2508.395</v>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
@@ -2863,13 +2863,13 @@
         <v>3061.556</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>2867.791</v>
+        <v>3480.102</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>6122.045</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>3174.638</v>
+        <v>2936.036</v>
       </c>
       <c r="L8" t="inlineStr"/>
     </row>
@@ -2903,13 +2903,13 @@
         <v>2661.555</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>2865.518</v>
+        <v>3397.829</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>3667.782</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>2113.596</v>
+        <v>1891.74</v>
       </c>
       <c r="L9" t="inlineStr"/>
     </row>
@@ -2943,13 +2943,13 @@
         <v>2235.628</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>3016.762</v>
+        <v>3463.887</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>8964.673000000001</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>8982.569</v>
+        <v>8968.51</v>
       </c>
       <c r="L10" t="inlineStr"/>
     </row>
@@ -2983,13 +2983,13 @@
         <v>939.573</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>1312.081</v>
+        <v>1499.996</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>4054.36</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>4107.195</v>
+        <v>4109.287</v>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
@@ -3023,13 +3023,13 @@
         <v>787.827</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>952.566</v>
+        <v>1110.132</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>2424.419</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>2318.077</v>
+        <v>2292.888</v>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
@@ -3063,13 +3063,13 @@
         <v>777.678</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>841.212</v>
+        <v>996.748</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1465.633</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>1155.567</v>
+        <v>1103.606</v>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
@@ -3103,13 +3103,13 @@
         <v>697.468</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>1640.405</v>
+        <v>1779.898</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>6812.267</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>7587.009</v>
+        <v>7698.729</v>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
@@ -3143,13 +3143,13 @@
         <v>677.96</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>1014.756</v>
+        <v>1150.348</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1509.059</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>769.27</v>
+        <v>718.367</v>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
@@ -3183,13 +3183,13 @@
         <v>657.741</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>782.0599999999999</v>
+        <v>913.6079999999999</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>2246.368</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>1626.919</v>
+        <v>1598.149</v>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
@@ -3223,13 +3223,13 @@
         <v>597.723</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>1018.817</v>
+        <v>1138.361</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>5017.485</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>4151.76</v>
+        <v>4187.996</v>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
@@ -3263,13 +3263,13 @@
         <v>530.367</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>424.294</v>
+        <v>530.367</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>413.686</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>53.037</v>
+        <v>0</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -3307,13 +3307,13 @@
         <v>418.481</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>984.242</v>
+        <v>1067.938</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>4087.36</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>4552.206</v>
+        <v>4619.238</v>
       </c>
       <c r="L19" t="inlineStr"/>
     </row>
@@ -3347,13 +3347,13 @@
         <v>406.554</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>600.601</v>
+        <v>681.9109999999999</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>827.372</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>386.074</v>
+        <v>353.75</v>
       </c>
       <c r="L20" t="inlineStr"/>
     </row>
@@ -3387,13 +3387,13 @@
         <v>356.026</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>386.863</v>
+        <v>458.068</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>717.511</v>
+        <v>698.304</v>
       </c>
       <c r="L21" t="inlineStr"/>
     </row>
@@ -3427,13 +3427,13 @@
         <v>356.026</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>386.863</v>
+        <v>458.068</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>717.511</v>
+        <v>698.304</v>
       </c>
       <c r="L22" t="inlineStr"/>
     </row>
@@ -3467,13 +3467,13 @@
         <v>279.968</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>721.438</v>
+        <v>777.432</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>3045.591</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>3327.504</v>
+        <v>3378.951</v>
       </c>
       <c r="L23" t="inlineStr"/>
     </row>
@@ -3507,13 +3507,13 @@
         <v>265.183</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>212.146</v>
+        <v>265.183</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>206.842</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>26.519</v>
+        <v>0</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -3551,13 +3551,13 @@
         <v>265.183</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>212.146</v>
+        <v>265.183</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>206.842</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>26.519</v>
+        <v>0</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -3595,13 +3595,13 @@
         <v>265.183</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>212.146</v>
+        <v>265.183</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>206.842</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>26.519</v>
+        <v>0</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -3639,13 +3639,13 @@
         <v>265.183</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>212.146</v>
+        <v>265.183</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>206.842</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>26.519</v>
+        <v>0</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -3683,13 +3683,13 @@
         <v>265.183</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>212.146</v>
+        <v>265.183</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>206.842</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>26.519</v>
+        <v>0</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -3727,13 +3727,13 @@
         <v>265.183</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>212.146</v>
+        <v>265.183</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>206.842</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>26.519</v>
+        <v>0</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -3771,13 +3771,13 @@
         <v>212.712</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>603.782</v>
+        <v>646.325</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>3025.502</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>3488.909</v>
+        <v>3551.253</v>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
@@ -3811,13 +3811,13 @@
         <v>211.641</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>587.37</v>
+        <v>629.698</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>2745.05</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>3087.994</v>
+        <v>3140.667</v>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
@@ -3851,13 +3851,13 @@
         <v>210.014</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>516.0309999999999</v>
+        <v>558.034</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>2266.489</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>2549.288</v>
+        <v>2588.784</v>
       </c>
       <c r="L32" t="inlineStr"/>
     </row>
@@ -3891,13 +3891,13 @@
         <v>141.83</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>403.239</v>
+        <v>431.605</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>2023.697</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>2333.427</v>
+        <v>2375.137</v>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
@@ -3931,13 +3931,13 @@
         <v>141.83</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>403.239</v>
+        <v>431.605</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>2023.697</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>2333.427</v>
+        <v>2375.137</v>
       </c>
       <c r="L34" t="inlineStr"/>
     </row>
@@ -3971,13 +3971,13 @@
         <v>141.829</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>403.238</v>
+        <v>431.604</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>2023.697</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>2333.428</v>
+        <v>2375.138</v>
       </c>
       <c r="L35" t="inlineStr"/>
     </row>
@@ -4011,13 +4011,13 @@
         <v>141.184</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>382.577</v>
+        <v>410.814</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>1843.427</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>2107.899</v>
+        <v>2144.141</v>
       </c>
       <c r="L36" t="inlineStr"/>
     </row>
@@ -4051,13 +4051,13 @@
         <v>140.758</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>386.076</v>
+        <v>414.228</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>1743.247</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>1933.621</v>
+        <v>1965.694</v>
       </c>
       <c r="L37" t="inlineStr"/>
     </row>
@@ -4091,13 +4091,13 @@
         <v>140.693</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>383.97</v>
+        <v>412.108</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>1723.157</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>1911.093</v>
+        <v>1942.713</v>
       </c>
       <c r="L38" t="inlineStr"/>
     </row>
@@ -4131,13 +4131,13 @@
         <v>140.629</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>381.865</v>
+        <v>409.991</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>1703.067</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>1888.565</v>
+        <v>1919.729</v>
       </c>
       <c r="L39" t="inlineStr"/>
     </row>
@@ -4171,13 +4171,13 @@
         <v>140.475</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>359.761</v>
+        <v>387.856</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1643.065</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>1859.911</v>
+        <v>1890.242</v>
       </c>
       <c r="L40" t="inlineStr"/>
     </row>
@@ -4211,13 +4211,13 @@
         <v>140.475</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>374.954</v>
+        <v>403.049</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>1660.745</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>1837.384</v>
+        <v>1867.167</v>
       </c>
       <c r="L41" t="inlineStr"/>
     </row>
@@ -4251,13 +4251,13 @@
         <v>140.41</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>372.847</v>
+        <v>400.929</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1640.656</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>1814.86</v>
+        <v>1844.187</v>
       </c>
       <c r="L42" t="inlineStr"/>
     </row>
@@ -4291,13 +4291,13 @@
         <v>140.41</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>357.61</v>
+        <v>385.692</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>1622.976</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>1837.45</v>
+        <v>1867.335</v>
       </c>
       <c r="L43" t="inlineStr"/>
     </row>
@@ -4331,13 +4331,13 @@
         <v>140.41</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>357.61</v>
+        <v>385.692</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>1622.976</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>1837.45</v>
+        <v>1867.335</v>
       </c>
       <c r="L44" t="inlineStr"/>
     </row>
@@ -4371,13 +4371,13 @@
         <v>140.409</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>357.609</v>
+        <v>385.691</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1622.976</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>1837.451</v>
+        <v>1867.336</v>
       </c>
       <c r="L45" t="inlineStr"/>
     </row>
@@ -4411,13 +4411,13 @@
         <v>139.623</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>362.011</v>
+        <v>389.935</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>1442.705</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>1518.393</v>
+        <v>1540.567</v>
       </c>
       <c r="L46" t="inlineStr"/>
     </row>
@@ -4451,13 +4451,13 @@
         <v>139.557</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>359.887</v>
+        <v>387.799</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>1422.616</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>1495.896</v>
+        <v>1517.604</v>
       </c>
       <c r="L47" t="inlineStr"/>
     </row>
@@ -4491,13 +4491,13 @@
         <v>139.557</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>359.887</v>
+        <v>387.799</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1422.616</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>1495.896</v>
+        <v>1517.604</v>
       </c>
       <c r="L48" t="inlineStr"/>
     </row>
@@ -4531,13 +4531,13 @@
         <v>139.493</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>328.08</v>
+        <v>355.978</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>1362.453</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>1517.402</v>
+        <v>1539.746</v>
       </c>
       <c r="L49" t="inlineStr"/>
     </row>
@@ -4571,13 +4571,13 @@
         <v>138.989</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>337.727</v>
+        <v>365.525</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>1257.613</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>1303.301</v>
+        <v>1320.424</v>
       </c>
       <c r="L50" t="inlineStr"/>
     </row>
@@ -4611,13 +4611,13 @@
         <v>137.26</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>270.904</v>
+        <v>298.356</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>887.725</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>715.107</v>
+        <v>718.3200000000001</v>
       </c>
       <c r="L51" t="inlineStr"/>
     </row>
@@ -4651,13 +4651,13 @@
         <v>136.379</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>234.022</v>
+        <v>261.298</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>576.775</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>419.962</v>
+        <v>416.062</v>
       </c>
       <c r="L52" t="inlineStr"/>
     </row>
@@ -4691,13 +4691,13 @@
         <v>135.518</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>200.2</v>
+        <v>227.303</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>275.79</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>128.691</v>
+        <v>117.916</v>
       </c>
       <c r="L53" t="inlineStr"/>
     </row>
@@ -4731,13 +4731,13 @@
         <v>135.518</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>200.2</v>
+        <v>227.303</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>275.79</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>128.691</v>
+        <v>117.916</v>
       </c>
       <c r="L54" t="inlineStr"/>
     </row>
@@ -4771,13 +4771,13 @@
         <v>135.517</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>200.199</v>
+        <v>227.303</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>275.79</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>128.692</v>
+        <v>117.916</v>
       </c>
       <c r="L55" t="inlineStr"/>
     </row>
@@ -4811,13 +4811,13 @@
         <v>72.57299999999999</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>267.015</v>
+        <v>281.529</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>1560.564</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>1725.561</v>
+        <v>1759.506</v>
       </c>
       <c r="L56" t="inlineStr"/>
     </row>
@@ -4851,13 +4851,13 @@
         <v>72.283</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>255.113</v>
+        <v>269.57</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1462.795</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>1628.537</v>
+        <v>1660.105</v>
       </c>
       <c r="L57" t="inlineStr"/>
     </row>
@@ -4891,13 +4891,13 @@
         <v>71.366</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>221.15</v>
+        <v>235.423</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1167.21</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>1317.142</v>
+        <v>1341.504</v>
       </c>
       <c r="L58" t="inlineStr"/>
     </row>
@@ -4931,13 +4931,13 @@
         <v>71.309</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>216.013</v>
+        <v>230.275</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1172.164</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>1302.234</v>
+        <v>1326.211</v>
       </c>
       <c r="L59" t="inlineStr"/>
     </row>
@@ -4971,13 +4971,13 @@
         <v>71.03400000000001</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>205.588</v>
+        <v>219.795</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1048.871</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>1208.103</v>
+        <v>1229.778</v>
       </c>
       <c r="L60" t="inlineStr"/>
     </row>
@@ -5011,13 +5011,13 @@
         <v>70.947</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L61" t="inlineStr"/>
     </row>
@@ -5051,13 +5051,13 @@
         <v>70.947</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L62" t="inlineStr"/>
     </row>
@@ -5091,13 +5091,13 @@
         <v>70.947</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L63" t="inlineStr"/>
     </row>
@@ -5131,13 +5131,13 @@
         <v>70.947</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L64" t="inlineStr"/>
     </row>
@@ -5171,13 +5171,13 @@
         <v>70.947</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L65" t="inlineStr"/>
     </row>
@@ -5211,13 +5211,13 @@
         <v>70.947</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L66" t="inlineStr"/>
     </row>
@@ -5251,13 +5251,13 @@
         <v>70.947</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L67" t="inlineStr"/>
     </row>
@@ -5291,13 +5291,13 @@
         <v>70.947</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L68" t="inlineStr"/>
     </row>
@@ -5331,13 +5331,13 @@
         <v>70.947</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L69" t="inlineStr"/>
     </row>
@@ -5371,13 +5371,13 @@
         <v>70.947</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L70" t="inlineStr"/>
     </row>
@@ -5411,13 +5411,13 @@
         <v>70.947</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L71" t="inlineStr"/>
     </row>
@@ -5451,13 +5451,13 @@
         <v>70.947</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>202.695</v>
+        <v>216.885</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L72" t="inlineStr"/>
     </row>
@@ -5491,13 +5491,13 @@
         <v>70.947</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>202.695</v>
+        <v>216.885</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L73" t="inlineStr"/>
     </row>
@@ -5531,13 +5531,13 @@
         <v>70.947</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L74" t="inlineStr"/>
     </row>
@@ -5571,13 +5571,13 @@
         <v>70.947</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>202.695</v>
+        <v>216.885</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L75" t="inlineStr"/>
     </row>
@@ -5611,13 +5611,13 @@
         <v>70.947</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>202.695</v>
+        <v>216.885</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L76" t="inlineStr"/>
     </row>
@@ -5651,13 +5651,13 @@
         <v>70.947</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>202.695</v>
+        <v>216.885</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L77" t="inlineStr"/>
     </row>
@@ -5691,13 +5691,13 @@
         <v>70.947</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>202.695</v>
+        <v>216.885</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L78" t="inlineStr"/>
     </row>
@@ -5731,13 +5731,13 @@
         <v>70.947</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L79" t="inlineStr"/>
     </row>
@@ -5771,13 +5771,13 @@
         <v>70.947</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>202.696</v>
+        <v>216.886</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>1021.893</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>1177.943</v>
+        <v>1199.02</v>
       </c>
       <c r="L80" t="inlineStr"/>
     </row>
@@ -5811,13 +5811,13 @@
         <v>70.88200000000001</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>200.542</v>
+        <v>214.719</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>1001.804</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>1155.484</v>
+        <v>1176.117</v>
       </c>
       <c r="L81" t="inlineStr"/>
     </row>
@@ -5851,13 +5851,13 @@
         <v>70.592</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>196.081</v>
+        <v>210.199</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>946.758</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>1046.845</v>
+        <v>1064.85</v>
       </c>
       <c r="L82" t="inlineStr"/>
     </row>
@@ -5891,13 +5891,13 @@
         <v>70.53</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>210.627</v>
+        <v>224.733</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>972.247</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>1000.474</v>
+        <v>1017.262</v>
       </c>
       <c r="L83" t="inlineStr"/>
     </row>
@@ -5931,13 +5931,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>179.88</v>
+        <v>193.928</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>929.956</v>
+        <v>945.122</v>
       </c>
       <c r="L84" t="inlineStr"/>
     </row>
@@ -5971,13 +5971,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>179.88</v>
+        <v>193.928</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>929.956</v>
+        <v>945.122</v>
       </c>
       <c r="L85" t="inlineStr"/>
     </row>
@@ -6011,13 +6011,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>179.88</v>
+        <v>193.928</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>929.956</v>
+        <v>945.122</v>
       </c>
       <c r="L86" t="inlineStr"/>
     </row>
@@ -6051,13 +6051,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>179.88</v>
+        <v>193.928</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>929.956</v>
+        <v>945.122</v>
       </c>
       <c r="L87" t="inlineStr"/>
     </row>
@@ -6091,13 +6091,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>179.88</v>
+        <v>193.928</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>929.956</v>
+        <v>945.122</v>
       </c>
       <c r="L88" t="inlineStr"/>
     </row>
@@ -6131,13 +6131,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>179.879</v>
+        <v>193.927</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>929.957</v>
+        <v>945.123</v>
       </c>
       <c r="L89" t="inlineStr"/>
     </row>
@@ -6171,13 +6171,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>179.879</v>
+        <v>193.927</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>929.957</v>
+        <v>945.123</v>
       </c>
       <c r="L90" t="inlineStr"/>
     </row>
@@ -6211,13 +6211,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>179.879</v>
+        <v>193.927</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>929.957</v>
+        <v>945.123</v>
       </c>
       <c r="L91" t="inlineStr"/>
     </row>
@@ -6251,13 +6251,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>179.88</v>
+        <v>193.928</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>929.956</v>
+        <v>945.122</v>
       </c>
       <c r="L92" t="inlineStr"/>
     </row>
@@ -6291,13 +6291,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>179.88</v>
+        <v>193.928</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>929.956</v>
+        <v>945.122</v>
       </c>
       <c r="L93" t="inlineStr"/>
     </row>
@@ -6331,13 +6331,13 @@
         <v>70.23699999999999</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>179.88</v>
+        <v>193.928</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>821.533</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>929.956</v>
+        <v>945.122</v>
       </c>
       <c r="L94" t="inlineStr"/>
     </row>
@@ -6371,13 +6371,13 @@
         <v>70.173</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>177.729</v>
+        <v>191.764</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>801.444</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>907.494</v>
+        <v>922.2140000000001</v>
       </c>
       <c r="L95" t="inlineStr"/>
     </row>
@@ -6411,13 +6411,13 @@
         <v>69.86</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>168.207</v>
+        <v>182.179</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>728.371</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>797.71</v>
+        <v>809.7910000000001</v>
       </c>
       <c r="L96" t="inlineStr"/>
     </row>
@@ -6451,13 +6451,13 @@
         <v>69.81100000000001</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>181.005</v>
+        <v>194.967</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>721.353</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>759.197</v>
+        <v>770.284</v>
       </c>
       <c r="L97" t="inlineStr"/>
     </row>
@@ -6491,13 +6491,13 @@
         <v>69.81100000000001</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>181.005</v>
+        <v>194.967</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>721.353</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>759.197</v>
+        <v>770.284</v>
       </c>
       <c r="L98" t="inlineStr"/>
     </row>
@@ -6531,13 +6531,13 @@
         <v>69.81100000000001</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>181.005</v>
+        <v>194.967</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>721.353</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>759.197</v>
+        <v>770.284</v>
       </c>
       <c r="L99" t="inlineStr"/>
     </row>
@@ -6571,13 +6571,13 @@
         <v>69.81100000000001</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>181.005</v>
+        <v>194.967</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>721.353</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>759.197</v>
+        <v>770.284</v>
       </c>
       <c r="L100" t="inlineStr"/>
     </row>
@@ -6611,13 +6611,13 @@
         <v>69.81100000000001</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>181.004</v>
+        <v>194.966</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>721.353</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>759.198</v>
+        <v>770.285</v>
       </c>
       <c r="L101" t="inlineStr"/>
     </row>
@@ -6651,13 +6651,13 @@
         <v>69.81100000000001</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>181.004</v>
+        <v>194.966</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>721.353</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>759.198</v>
+        <v>770.285</v>
       </c>
       <c r="L102" t="inlineStr"/>
     </row>
@@ -6691,13 +6691,13 @@
         <v>69.747</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>164.041</v>
+        <v>177.99</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>681.226</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>758.701</v>
+        <v>769.872</v>
       </c>
       <c r="L103" t="inlineStr"/>
     </row>
@@ -6731,13 +6731,13 @@
         <v>69.747</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>178.883</v>
+        <v>192.832</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>701.2619999999999</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>736.698</v>
+        <v>747.3200000000001</v>
       </c>
       <c r="L104" t="inlineStr"/>
     </row>
@@ -6771,13 +6771,13 @@
         <v>69.747</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>164.04</v>
+        <v>177.989</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>681.226</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>758.702</v>
+        <v>769.873</v>
       </c>
       <c r="L105" t="inlineStr"/>
     </row>
@@ -6811,13 +6811,13 @@
         <v>69.527</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>169.928</v>
+        <v>183.833</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>638.851</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>662.896</v>
+        <v>671.6900000000001</v>
       </c>
       <c r="L106" t="inlineStr"/>
     </row>
@@ -6851,13 +6851,13 @@
         <v>69.527</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>169.927</v>
+        <v>183.832</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>638.851</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>662.896</v>
+        <v>671.691</v>
       </c>
       <c r="L107" t="inlineStr"/>
     </row>
@@ -6891,13 +6891,13 @@
         <v>69.527</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>169.927</v>
+        <v>183.832</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>638.851</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>662.896</v>
+        <v>671.691</v>
       </c>
       <c r="L108" t="inlineStr"/>
     </row>
@@ -6931,13 +6931,13 @@
         <v>69.5</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>167.317</v>
+        <v>181.217</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>720.927</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>654.372</v>
+        <v>662.871</v>
       </c>
       <c r="L109" t="inlineStr"/>
     </row>
@@ -6971,13 +6971,13 @@
         <v>69.14</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>144.069</v>
+        <v>157.897</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>584.207</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>546.828</v>
+        <v>552.854</v>
       </c>
       <c r="L110" t="inlineStr"/>
     </row>
@@ -7011,13 +7011,13 @@
         <v>68.946</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>148.248</v>
+        <v>162.037</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>554.088</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>464.015</v>
+        <v>468.114</v>
       </c>
       <c r="L111" t="inlineStr"/>
     </row>
@@ -7051,13 +7051,13 @@
         <v>68.804</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>142.533</v>
+        <v>156.294</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>503.997</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>416.236</v>
+        <v>419.224</v>
       </c>
       <c r="L112" t="inlineStr"/>
     </row>
@@ -7091,13 +7091,13 @@
         <v>68.64</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>128.021</v>
+        <v>141.749</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>379.829</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>373.353</v>
+        <v>375.243</v>
       </c>
       <c r="L113" t="inlineStr"/>
     </row>
@@ -7131,13 +7131,13 @@
         <v>68.114</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>111.375</v>
+        <v>124.998</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>252.808</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>188.369</v>
+        <v>185.935</v>
       </c>
       <c r="L114" t="inlineStr"/>
     </row>
@@ -7171,13 +7171,13 @@
         <v>68.114</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>114.429</v>
+        <v>128.052</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>263.121</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>183.976</v>
+        <v>181.471</v>
       </c>
       <c r="L115" t="inlineStr"/>
     </row>
@@ -7211,13 +7211,13 @@
         <v>68.107</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>111.131</v>
+        <v>124.753</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>225.004</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>186.627</v>
+        <v>184.11</v>
       </c>
       <c r="L116" t="inlineStr"/>
     </row>
@@ -7251,13 +7251,13 @@
         <v>67.97199999999999</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>108.319</v>
+        <v>121.913</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>213.03</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>136.59</v>
+        <v>132.907</v>
       </c>
       <c r="L117" t="inlineStr"/>
     </row>
@@ -7291,13 +7291,13 @@
         <v>67.97199999999999</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>108.318</v>
+        <v>121.912</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>213.03</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>136.591</v>
+        <v>132.908</v>
       </c>
       <c r="L118" t="inlineStr"/>
     </row>
@@ -7331,13 +7331,13 @@
         <v>67.97199999999999</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>108.572</v>
+        <v>122.166</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>213.03</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>136.305</v>
+        <v>132.65</v>
       </c>
       <c r="L119" t="inlineStr"/>
     </row>
@@ -7371,13 +7371,13 @@
         <v>67.759</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>100.1</v>
+        <v>113.652</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K120" s="2" t="n">
-        <v>64.346</v>
+        <v>58.959</v>
       </c>
       <c r="L120" t="inlineStr"/>
     </row>
@@ -7411,13 +7411,13 @@
         <v>67.759</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>100.1</v>
+        <v>113.652</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>64.346</v>
+        <v>58.959</v>
       </c>
       <c r="L121" t="inlineStr"/>
     </row>
@@ -7451,13 +7451,13 @@
         <v>67.759</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>100.1</v>
+        <v>113.652</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>64.346</v>
+        <v>58.959</v>
       </c>
       <c r="L122" t="inlineStr"/>
     </row>
@@ -7491,13 +7491,13 @@
         <v>67.759</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>100.1</v>
+        <v>113.652</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>64.346</v>
+        <v>58.959</v>
       </c>
       <c r="L123" t="inlineStr"/>
     </row>
@@ -7531,13 +7531,13 @@
         <v>67.759</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>100.099</v>
+        <v>113.651</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>64.34699999999999</v>
+        <v>58.96</v>
       </c>
       <c r="L124" t="inlineStr"/>
     </row>
@@ -7571,13 +7571,13 @@
         <v>67.759</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>100.099</v>
+        <v>113.651</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K125" s="2" t="n">
-        <v>64.34699999999999</v>
+        <v>58.96</v>
       </c>
       <c r="L125" t="inlineStr"/>
     </row>
@@ -7611,13 +7611,13 @@
         <v>67.759</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>100.099</v>
+        <v>113.651</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K126" s="2" t="n">
-        <v>64.34699999999999</v>
+        <v>58.96</v>
       </c>
       <c r="L126" t="inlineStr"/>
     </row>
@@ -7651,13 +7651,13 @@
         <v>67.759</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>100.099</v>
+        <v>113.651</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K127" s="2" t="n">
-        <v>64.34699999999999</v>
+        <v>58.96</v>
       </c>
       <c r="L127" t="inlineStr"/>
     </row>
@@ -7691,13 +7691,13 @@
         <v>67.759</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>100.099</v>
+        <v>113.651</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K128" s="2" t="n">
-        <v>64.34699999999999</v>
+        <v>58.96</v>
       </c>
       <c r="L128" t="inlineStr"/>
     </row>
@@ -7731,13 +7731,13 @@
         <v>67.759</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>100.099</v>
+        <v>113.651</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K129" s="2" t="n">
-        <v>64.34699999999999</v>
+        <v>58.96</v>
       </c>
       <c r="L129" t="inlineStr"/>
     </row>
@@ -7771,13 +7771,13 @@
         <v>67.759</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>100.1</v>
+        <v>113.652</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K130" s="2" t="n">
-        <v>64.346</v>
+        <v>58.959</v>
       </c>
       <c r="L130" t="inlineStr"/>
     </row>
@@ -7811,13 +7811,13 @@
         <v>67.759</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>100.1</v>
+        <v>113.652</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K131" s="2" t="n">
-        <v>64.346</v>
+        <v>58.959</v>
       </c>
       <c r="L131" t="inlineStr"/>
     </row>
@@ -7851,13 +7851,13 @@
         <v>67.759</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>100.1</v>
+        <v>113.652</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>64.346</v>
+        <v>58.959</v>
       </c>
       <c r="L132" t="inlineStr"/>
     </row>
@@ -7891,13 +7891,13 @@
         <v>67.759</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>100.1</v>
+        <v>113.652</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>137.895</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>64.346</v>
+        <v>58.959</v>
       </c>
       <c r="L133" t="inlineStr"/>
     </row>
@@ -7937,7 +7937,7 @@
         <v>540.143</v>
       </c>
       <c r="K134" s="2" t="n">
-        <v>565.776</v>
+        <v>579.018</v>
       </c>
       <c r="L134" t="inlineStr"/>
     </row>
@@ -7977,7 +7977,7 @@
         <v>213.326</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>192.327</v>
+        <v>196.854</v>
       </c>
       <c r="L135" t="inlineStr"/>
     </row>
@@ -8044,7 +8044,7 @@
         <v>1826.525</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1552.786</v>
+        <v>440.718</v>
       </c>
     </row>
     <row r="4">
@@ -8057,7 +8057,7 @@
         <v>5898.341</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>11230.422</v>
+        <v>9607.509</v>
       </c>
     </row>
     <row r="5">
@@ -8070,7 +8070,7 @@
         <v>783.068</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1535.083</v>
+        <v>623.422</v>
       </c>
     </row>
     <row r="6">
@@ -8109,7 +8109,7 @@
         <v>11.862</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>16807.94</v>
+        <v>20454.582</v>
       </c>
     </row>
     <row r="9">
@@ -8135,7 +8135,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>4080.378</v>
+        <v>4198.909</v>
       </c>
     </row>
     <row r="11">
@@ -8148,7 +8148,7 @@
         <v>0</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>197.551</v>
+        <v>79.02</v>
       </c>
     </row>
     <row r="12">
@@ -8378,7 +8378,7 @@
         <v>75.13500000000001</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>23.609</v>
+        <v>17.158</v>
       </c>
     </row>
     <row r="30">
@@ -8391,7 +8391,7 @@
         <v>128.363</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>308.201</v>
+        <v>314.652</v>
       </c>
     </row>
     <row r="31">
@@ -8443,7 +8443,7 @@
         <v>0</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>154.174</v>
+        <v>158.642</v>
       </c>
     </row>
     <row r="35">
@@ -8456,7 +8456,7 @@
         <v>0</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>7.446</v>
+        <v>2.978</v>
       </c>
     </row>
     <row r="36">
@@ -8851,28 +8851,28 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Prosthesis profile SWNurs 3.6%, SWDoc 29.5%, SWAllied 11.1%, Prostheses 54.3%, MS 1.5%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Prosthesis profile SWNurs 3.1%, SWDoc 26.0%, SWAllied 9.8%, Prostheses 59.8%, MS 1.4%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Dental profile SWNurs 8.1%, SWDoc 41.8%, SWAllied 2.2%, Prostheses 1.9%, MS 7.4%, GS 0.3%, Depreciation 2.6%, OHF 32.7%, OHDepreciation 0.7%, OHC 2.3%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Dental profile SWNurs 8.0%, SWDoc 42.7%, SWAllied 2.2%, MS 7.5%, GS 0.3%, Depreciation 2.6%, OHF 33.6%, OHDepreciation 0.7%, OHC 2.3%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Imaging profile SWNurs 7.4%, SWDoc 40.7%, SWAllied 4.1%, Prostheses 14.1%, MS 6.4%, Depreciation 2.1%, OHF 25.2%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Imaging profile SWNurs 10.4%, SWDoc 57.6%, SWAllied 5.8%, MS 9.0%, Depreciation 3.0%, OHF 14.2%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Anaesthesia profile SWNurs 9.7%, SWDoc 53.8%, Pharmacy 6.6%, Prostheses 18.6%, MS 8.4%, Depreciation 2.8%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Anaesthesia profile SWNurs 17.2%, SWDoc 57.1%, Pharmacy 11.8%, MS 8.9%, Depreciation 5.0%</t>
         </is>
       </c>
     </row>
@@ -8935,28 +8935,28 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Prosthesis profile SWNurs 3.1%, SWDoc 37.9%, SWAllied 7.9%, Prostheses 49.6%, MS 1.5%</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Prosthesis profile SWNurs 2.8%, SWDoc 33.7%, SWAllied 7.0%, Prostheses 55.2%, MS 1.3%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Dental profile SWNurs 6.1%, SWDoc 46.0%, SWAllied 1.7%, Prostheses 1.5%, MS 6.1%, GS 0.6%, Depreciation 2.4%, OHF 25.4%, OHDepreciation 0.6%, OHC 9.5%</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Dental profile SWNurs 6.1%, SWDoc 46.9%, SWAllied 1.7%, MS 6.2%, GS 0.6%, Depreciation 2.4%, OHF 26.1%, OHDepreciation 0.6%, OHC 9.4%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Imaging profile SWNurs 6.1%, SWDoc 49.1%, SWAllied 3.4%, Prostheses 12.1%, MS 5.8%, Depreciation 2.2%, OHF 21.4%</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Imaging profile SWNurs 8.1%, SWDoc 65.4%, SWAllied 4.5%, MS 7.7%, Depreciation 2.9%, OHF 11.4%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Anaesthesia profile SWNurs 7.7%, SWDoc 61.6%, Pharmacy 5.6%, Prostheses 15.1%, MS 7.3%, Depreciation 2.7%</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Anaesthesia profile SWNurs 13.4%, SWDoc 64.5%, Pharmacy 9.8%, MS 7.6%, Depreciation 4.7%</t>
         </is>
       </c>
     </row>
@@ -9362,28 +9362,28 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Prosthesis profile SWNurs 2.7%, SWDoc 30.2%, SWAllied 6.9%, Prostheses 58.9%, MS 1.3%</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Prosthesis profile SWNurs 2.4%, SWDoc 26.4%, SWAllied 6.0%, Prostheses 64.1%, MS 1.1%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Dental profile SWNurs 5.9%, SWDoc 41.3%, SWAllied 1.7%, Prostheses 2.0%, MS 6.0%, Depreciation 2.2%, OHF 26.1%, OHDepreciation 0.6%, OHC 14.2%</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Dental profile SWNurs 5.9%, SWDoc 42.4%, SWAllied 1.7%, MS 6.1%, Depreciation 2.2%, OHF 26.9%, OHDepreciation 0.6%, OHC 14.2%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Imaging profile SWNurs 6.0%, SWDoc 44.5%, SWAllied 3.4%, Prostheses 16.2%, MS 5.7%, Depreciation 1.9%, OHF 22.2%</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Imaging profile SWNurs 8.5%, SWDoc 63.2%, SWAllied 4.8%, MS 8.1%, Depreciation 2.8%, OHF 12.6%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Anaesthesia profile SWNurs 7.7%, SWDoc 56.8%, Pharmacy 5.0%, Prostheses 20.7%, MS 7.3%, Depreciation 2.5%</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Anaesthesia profile SWNurs 14.3%, SWDoc 63.6%, Pharmacy 9.3%, MS 8.2%, Depreciation 4.6%</t>
         </is>
       </c>
     </row>
@@ -9530,28 +9530,28 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Prosthesis profile SWNurs 3.7%, SWDoc 27.0%, SWAllied 5.6%, Prostheses 62.0%, MS 1.7%</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Prosthesis profile SWNurs 3.2%, SWDoc 23.4%, SWAllied 4.9%, Prostheses 67.1%, MS 1.5%</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Dental profile SWNurs 7.0%, SWDoc 31.7%, SWAllied 1.9%, Prostheses 1.8%, MS 6.8%, GS 0.2%, Depreciation 2.4%, OHF 30.4%, OHDepreciation 0.7%, OHC 17.1%</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Dental profile SWNurs 7.0%, SWDoc 32.4%, SWAllied 1.8%, MS 6.9%, GS 0.2%, Depreciation 2.4%, OHF 31.4%, OHDepreciation 0.6%, OHC 17.1%</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Imaging profile SWNurs 7.5%, SWDoc 36.2%, SWAllied 4.0%, Prostheses 15.6%, MS 6.9%, Depreciation 2.3%, OHF 27.5%</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Imaging profile SWNurs 11.1%, SWDoc 53.4%, SWAllied 5.9%, MS 10.1%, Depreciation 3.4%, OHF 16.2%</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Anaesthesia profile SWNurs 10.3%, SWDoc 49.5%, Pharmacy 6.4%, Prostheses 21.3%, MS 9.4%, Depreciation 3.2%</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Anaesthesia profile SWNurs 18.6%, SWDoc 53.8%, Pharmacy 11.6%, MS 10.2%, Depreciation 5.8%</t>
         </is>
       </c>
     </row>
@@ -9614,28 +9614,28 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Prosthesis profile SWNurs 4.4%, SWDoc 30.8%, SWAllied 8.8%, Prostheses 54.7%, MS 1.3%</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Prosthesis profile SWNurs 3.8%, SWDoc 27.1%, SWAllied 7.7%, Prostheses 60.2%, MS 1.1%</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Dental profile SWNurs 9.2%, SWDoc 40.6%, SWAllied 2.3%, Prostheses 1.8%, MS 5.8%, Depreciation 2.7%, OHF 36.3%, OHDepreciation 0.7%, OHC 0.7%</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Dental profile SWNurs 9.1%, SWDoc 41.4%, SWAllied 2.2%, MS 5.9%, Depreciation 2.7%, OHF 37.2%, OHDepreciation 0.7%, OHC 0.7%</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Imaging profile SWNurs 8.3%, SWDoc 39.4%, SWAllied 4.1%, Prostheses 13.1%, MS 5.0%, Depreciation 2.2%, OHF 27.8%</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Imaging profile SWNurs 11.9%, SWDoc 56.2%, SWAllied 5.8%, MS 7.1%, Depreciation 3.1%, OHF 15.9%</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Anaesthesia profile SWNurs 11.5%, SWDoc 54.2%, Pharmacy 6.5%, Prostheses 18.0%, MS 6.8%, Depreciation 3.0%</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Anaesthesia profile SWNurs 19.9%, SWDoc 56.5%, Pharmacy 11.3%, MS 7.1%, Depreciation 5.2%</t>
         </is>
       </c>
     </row>
@@ -9691,28 +9691,28 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Prosthesis profile SWNurs 6.9%, SWDoc 40.6%, SWAllied 1.7%, Prostheses 49.4%, MS 1.3%</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Prosthesis profile SWNurs 6.1%, SWDoc 36.2%, SWAllied 1.5%, Prostheses 55.0%, MS 1.2%</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Dental profile SWNurs 9.8%, SWDoc 36.2%, SWAllied 2.5%, Prostheses 1.1%, MS 4.1%, Depreciation 2.0%, OHF 36.0%, OHDepreciation 0.5%, OHC 7.8%</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Dental profile SWNurs 9.7%, SWDoc 36.8%, SWAllied 2.4%, MS 4.1%, Depreciation 2.0%, OHF 36.8%, OHDepreciation 0.5%, OHC 7.7%</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Imaging profile SWNurs 10.0%, SWDoc 39.4%, SWAllied 5.0%, Prostheses 9.0%, MS 3.9%, Depreciation 1.8%, OHF 30.9%</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Imaging profile SWNurs 13.8%, SWDoc 54.3%, SWAllied 6.9%, MS 5.4%, Depreciation 2.5%, OHF 17.1%</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Anaesthesia profile SWNurs 14.9%, SWDoc 58.3%, Pharmacy 5.1%, Prostheses 13.3%, MS 5.8%, Depreciation 2.6%</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Anaesthesia profile SWNurs 24.3%, SWDoc 57.3%, Pharmacy 8.3%, MS 5.7%, Depreciation 4.3%</t>
         </is>
       </c>
     </row>
@@ -9817,28 +9817,28 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Prosthesis profile SWNurs 5.8%, SWDoc 33.0%, SWAllied 10.0%, Prostheses 49.5%, MS 1.7%</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Prosthesis profile SWNurs 5.1%, SWDoc 29.4%, SWAllied 8.9%, Prostheses 55.1%, MS 1.5%</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Dental profile SWNurs 9.5%, SWDoc 33.9%, SWAllied 2.6%, Prostheses 1.3%, MS 6.0%, Depreciation 2.6%, OHF 36.5%, OHDepreciation 0.7%, OHC 6.8%</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Dental profile SWNurs 9.4%, SWDoc 34.5%, SWAllied 2.6%, MS 6.1%, Depreciation 2.6%, OHF 37.3%, OHDepreciation 0.7%, OHC 6.8%</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Imaging profile SWNurs 9.5%, SWDoc 36.2%, SWAllied 5.2%, Prostheses 10.2%, MS 5.7%, Depreciation 2.3%, OHF 30.8%</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Imaging profile SWNurs 13.3%, SWDoc 50.8%, SWAllied 7.3%, MS 8.0%, Depreciation 3.2%, OHF 17.3%</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Anaesthesia profile SWNurs 13.5%, SWDoc 51.4%, Pharmacy 9.3%, Prostheses 14.4%, MS 8.1%, Depreciation 3.3%</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Anaesthesia profile SWNurs 21.8%, SWDoc 49.9%, Pharmacy 15.1%, MS 7.8%, Depreciation 5.3%</t>
         </is>
       </c>
     </row>
@@ -9957,28 +9957,28 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Prosthesis profile SWNurs 4.8%, SWDoc 23.5%, SWAllied 14.0%, Prostheses 56.2%, MS 1.5%</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Prosthesis profile SWNurs 4.2%, SWDoc 20.6%, SWAllied 12.3%, Prostheses 61.6%, MS 1.3%</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Dental profile SWNurs 9.9%, SWDoc 30.3%, SWAllied 2.4%, Prostheses 1.8%, MS 6.7%, Depreciation 2.5%, OHF 38.7%, OHDepreciation 0.7%, OHC 7.1%</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Dental profile SWNurs 9.8%, SWDoc 31.0%, SWAllied 2.4%, MS 6.8%, Depreciation 2.5%, OHF 39.8%, OHDepreciation 0.7%, OHC 7.1%</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Imaging profile SWNurs 9.6%, SWDoc 31.5%, SWAllied 4.6%, Prostheses 14.2%, MS 6.1%, Depreciation 2.1%, OHF 31.8%</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Imaging profile SWNurs 14.4%, SWDoc 47.2%, SWAllied 7.0%, MS 9.2%, Depreciation 3.2%, OHF 19.0%</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Anaesthesia profile SWNurs 13.9%, SWDoc 45.6%, Pharmacy 8.0%, Prostheses 20.5%, MS 8.9%, Depreciation 3.1%</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Anaesthesia profile SWNurs 24.1%, SWDoc 47.5%, Pharmacy 13.8%, MS 9.2%, Depreciation 5.4%</t>
         </is>
       </c>
     </row>
@@ -10041,28 +10041,28 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Prosthesis profile SWNurs 3.5%, SWDoc 29.3%, SWAllied 13.4%, Prostheses 52.3%, MS 1.4%</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Prosthesis profile SWNurs 3.1%, SWDoc 25.9%, SWAllied 11.9%, Prostheses 57.8%, MS 1.3%</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Dental profile SWNurs 6.5%, SWDoc 33.9%, SWAllied 2.4%, Prostheses 1.5%, MS 5.6%, Depreciation 2.5%, OHF 39.5%, OHDepreciation 0.7%, OHC 7.4%</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Dental profile SWNurs 6.5%, SWDoc 34.6%, SWAllied 2.4%, MS 5.7%, Depreciation 2.5%, OHF 40.4%, OHDepreciation 0.7%, OHC 7.3%</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Imaging profile SWNurs 6.5%, SWDoc 36.1%, SWAllied 4.8%, Prostheses 12.1%, MS 5.3%, Depreciation 2.2%, OHF 33.1%</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Imaging profile SWNurs 9.5%, SWDoc 53.0%, SWAllied 7.0%, MS 7.8%, Depreciation 3.2%, OHF 19.5%</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Anaesthesia profile SWNurs 9.1%, SWDoc 50.4%, Pharmacy 13.1%, Prostheses 16.9%, MS 7.4%, Depreciation 3.1%</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Anaesthesia profile SWNurs 15.1%, SWDoc 50.4%, Pharmacy 21.9%, MS 7.4%, Depreciation 5.2%</t>
         </is>
       </c>
     </row>
@@ -10125,28 +10125,28 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Prosthesis profile SWNurs 4.8%, SWDoc 38.3%, SWAllied 9.5%, Prostheses 45.9%, MS 1.4%</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Prosthesis profile SWNurs 4.3%, SWDoc 34.4%, SWAllied 8.5%, Prostheses 51.5%, MS 1.3%</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Dental profile SWNurs 8.0%, SWDoc 39.7%, SWAllied 2.1%, Prostheses 1.2%, MS 5.1%, GS 0.3%, Depreciation 2.3%, OHF 34.5%, OHDepreciation 0.6%, OHC 6.1%</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Dental profile SWNurs 7.9%, SWDoc 40.3%, SWAllied 2.1%, MS 5.2%, GS 0.3%, Depreciation 2.3%, OHF 35.3%, OHDepreciation 0.6%, OHC 6.1%</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Imaging profile SWNurs 8.0%, SWDoc 42.3%, SWAllied 4.2%, Prostheses 9.5%, MS 4.8%, Depreciation 2.0%, OHF 29.1%</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Imaging profile SWNurs 10.9%, SWDoc 58.0%, SWAllied 5.8%, MS 6.6%, Depreciation 2.8%, OHF 15.9%</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Anaesthesia profile SWNurs 11.2%, SWDoc 59.6%, Pharmacy 6.2%, Prostheses 13.4%, MS 6.8%, Depreciation 2.9%</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Anaesthesia profile SWNurs 18.7%, SWDoc 59.5%, Pharmacy 10.3%, MS 6.8%, Depreciation 4.8%</t>
         </is>
       </c>
     </row>
@@ -10209,28 +10209,28 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Prosthesis profile SWNurs 4.7%, SWDoc 28.5%, SWAllied 13.6%, Prostheses 51.7%, MS 1.5%</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Prosthesis profile SWNurs 4.1%, SWDoc 25.3%, SWAllied 12.0%, Prostheses 57.2%, MS 1.3%</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Dental profile SWNurs 8.4%, SWDoc 32.0%, SWAllied 2.2%, Prostheses 1.5%, MS 5.7%, Depreciation 2.6%, OHF 40.3%, OHDepreciation 0.7%, OHC 6.7%</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Dental profile SWNurs 8.3%, SWDoc 32.6%, SWAllied 2.2%, MS 5.8%, Depreciation 2.5%, OHF 41.2%, OHDepreciation 0.7%, OHC 6.7%</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Imaging profile SWNurs 8.4%, SWDoc 34.2%, SWAllied 4.3%, Prostheses 11.6%, MS 5.4%, Depreciation 2.3%, OHF 33.9%</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Imaging profile SWNurs 12.3%, SWDoc 50.2%, SWAllied 6.4%, MS 7.9%, Depreciation 3.3%, OHF 19.9%</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Anaesthesia profile SWNurs 12.5%, SWDoc 51.0%, Pharmacy 7.7%, Prostheses 17.3%, MS 8.1%, Depreciation 3.4%</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Anaesthesia profile SWNurs 21.1%, SWDoc 51.8%, Pharmacy 13.1%, MS 8.2%, Depreciation 5.7%</t>
         </is>
       </c>
     </row>
@@ -10370,28 +10370,28 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Prosthesis profile SWNurs 3.9%, SWDoc 31.2%, SWAllied 17.5%, Prostheses 46.4%, MS 1.0%</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Prosthesis profile SWNurs 3.5%, SWDoc 27.9%, SWAllied 15.7%, Prostheses 52.0%, MS 0.9%</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Dental profile SWNurs 8.2%, SWDoc 40.7%, SWAllied 2.2%, Prostheses 1.5%, MS 4.4%, GS 0.0%, Depreciation 2.1%, OHF 34.8%, OHDepreciation 0.6%, OHC 5.5%</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Dental profile SWNurs 8.1%, SWDoc 41.5%, SWAllied 2.2%, MS 4.4%, GS 0.0%, Depreciation 2.1%, OHF 35.6%, OHDepreciation 0.6%, OHC 5.5%</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Imaging profile SWNurs 7.9%, SWDoc 42.0%, SWAllied 4.3%, Prostheses 11.7%, MS 4.0%, Depreciation 1.8%, OHF 28.3%</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Imaging profile SWNurs 11.1%, SWDoc 58.9%, SWAllied 6.1%, MS 5.6%, Depreciation 2.5%, OHF 15.9%</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Anaesthesia profile SWNurs 11.3%, SWDoc 59.9%, Pharmacy 3.8%, Prostheses 16.7%, MS 5.7%, Depreciation 2.6%</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Anaesthesia profile SWNurs 19.8%, SWDoc 63.1%, Pharmacy 6.7%, MS 6.0%, Depreciation 4.5%</t>
         </is>
       </c>
     </row>

</xml_diff>